<commit_message>
docs: sync roadmap, changelog, handoff, team brief, README; refresh features matrix
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/submission/GPTHub_features_matrix.xlsx
+++ b/docs/submission/GPTHub_features_matrix.xlsx
@@ -725,12 +725,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Deferred (wow candidate)</t>
+          <t>Implemented (WOW-1)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Запланирован как **Expert Council**: новый `task_type=DEEP_RESEARCH`, orchestrator внутри делает fan-out в 3 модели MWS (`strong` + `reasoning` + `doc`), собирает synthesis через `strong`, возвращает один ответ в один chat flow. Архитектурно не ломает «один запрос → один ответ».</t>
+          <t>**Expert Council**: `/research` или «глубокое исследование» → `task_type=DEEP_RESEARCH` → `apps/orchestrator/gpthub_orchestrator/council.py` делает параллельный fan-out в 3 MWS-модели (`gpt-hub-turbo` generalist, `gpt-hub-reasoning-or` reasoning, `gpt-hub-doc` doc-expert), каждая с собственной персоной, а затем `gpt-hub-strong` (glm-4.6-357b) синтезирует один финальный ответ в формате «суть → «что говорит совет экспертов» → практические рекомендации». CoT-очистка, partial-failure tolerant (≥2/3 веток), strong-only fallback, emergency composite если synthesis деградирует. Один `chat.completion` на выход. 29 unit-тестов (`test_council.py`) + live smoke через docker (171 s, 3/3 ветки, запись в LIVE_SMOKE.md 2026-04-11). Трейс: `{short_circuit:"expert_council", branches_ok:[...3 moderms...], synthesis_model, total_ms, fallback_used}`.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: WOW-3 PPTX generation (row 14) + Tavily toggle + full doc sync
- New `pptx_gen.py`: intent detection (RU/EN + /pptx /slides), JSON
  slide plan via gpt-hub-strong with retry, python-pptx builder,
  file storage + download endpoint GET /v1/files/pptx/{token}.
  52 unit tests in test_pptx_gen.py. Total: 234 tests passing.
- Classifier gains TaskType.PPTX_GENERATION; router adds fallback.
- Short-circuit wired in main.py between council and image-gen.
- Row 7 Tavily env vars confirmed in .env + running container.
- Full doc sync: ROADMAP (§0.2 row 14, §0.4 snapshot, §5 post-
  competition roadmap), CHANGELOG, README (234 tests, PPTX bullet),
  FEATURE_MATRIX (row 14 Implemented WOW-3), TEAM_BRIEF_RU,
  NEW_CHAT_HANDOFF_RU, LIVE_SMOKE (operator checklist for Step 6).
- Regenerated GPTHub_features_matrix.xlsx.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/submission/GPTHub_features_matrix.xlsx
+++ b/docs/submission/GPTHub_features_matrix.xlsx
@@ -747,12 +747,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Deferred (wow candidate)</t>
+          <t>Implemented (WOW-3)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Orchestrator-тул: классификатор ловит «сделай презентацию / /pptx» → strong-модель генерирует JSON slide plan → `python-pptx` собирает `.pptx` → возвращается base64 attachment + markdown preview. Зависимость `python-pptx`.</t>
+          <t>**PPTX generation**: `/pptx` или «сделай презентацию / build a deck» → `task_type=PPTX_GENERATION` → `apps/orchestrator/gpthub_orchestrator/pptx_gen.py` просит `gpt-hub-strong` (glm-4.6-357b) сгенерировать JSON slide plan (retry on parse failure), затем `python-pptx` собирает `.pptx` (title slide + bullet slides), файл сохраняется в `/tmp/gpthub_pptx/`, в ответ идёт markdown-ссылка на `GET /v1/files/pptx/{token}`. Один `chat.completion` на выход. 52 unit-теста (`test_pptx_gen.py`). Трейс: `{short_circuit:"pptx_generation", plan_model, slide_count, byte_size, plan_ms, build_ms, url}`.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: study onboarding path and submission diagrams; fix payload_log clip
</commit_message>
<xml_diff>
--- a/docs/submission/GPTHub_features_matrix.xlsx
+++ b/docs/submission/GPTHub_features_matrix.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Open WebUI → orchestrator `/v1/chat/completions` → LiteLLM alias `gpt-hub-turbo/strong` → MWS `mws-gpt-alpha` / `glm-4.6-357b`. Prompt precedence + `X-GPTHub-Trace`.</t>
+          <t>Open WebUI → orchestrator `/v1/chat/completions` → LiteLLM (по умолчанию `gpt-hub-turbo` → `mws-gpt-alpha`; другие task_type см. ряд 10). Prompt precedence + `X-GPTHub-Trace`.</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Включён через Open WebUI web search (`ENABLE_WEB_SEARCH=true`, `WEB_SEARCH_ENGINE=tavily`, `TAVILY_API_KEY`). Результаты приходят в сообщение, дальше общий orchestrator-путь.</t>
+          <t>Включён через Open WebUI web search (`ENABLE_WEB_SEARCH=true`, `WEB_SEARCH_ENGINE=tavily`, `TAVILY_API_KEY`). Обязательно **`BYPASS_WEB_SEARCH_EMBEDDING_AND_RETRIEVAL=true`** (или эквивалентный тумблер в Admin → Web Search): иначе WebUI пытается векторизовать сниппеты без embedding engine → ошибка и пустые источники. С bypass сниппеты **встраиваются в текст запроса** к orchestrator; **панель «источники»** может кратко показывать число находок, затем **«источники не найдены»**, потому что UI часто ждёт метаданные из пропущенного vector-пути — это **косметика**, не признак отсутствия поиска, если ответ по сути совпадает с новостями. Дальше — общий orchestrator-путь.</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>`apps/orchestrator/gpthub_orchestrator/memory/`: SQLite store (`store.py`), command parser (`commands.py`), MWS `qwen3-embedding-8b` client (`embeddings.py`), высокоуровневый сервис (`service.py`). Orchestrator ловит «запомни X / забудь X / что ты помнишь», сохраняет факты с эмбеддингом, при обычном запросе подмешивает top-K релевантных фактов как system-блок. Тесты: `test_memory_commands.py`, `test_memory_store.py`, `test_memory_service.py` (52 теста).</t>
+          <t>`apps/orchestrator/gpthub_orchestrator/memory/`: SQLite store (`store.py`), command parser (`commands.py`), MWS `qwen3-embedding-8b` client (`embeddings.py`), высокоуровневый сервис (`service.py`). Orchestrator ловит «запомни X / забудь X / что ты помнишь», сохраняет факты с эмбеддингом, при обычном запросе подмешивает top-K релевантных фактов как system-блок. Тесты: `test_memory_commands.py`, `test_memory_store.py`, `test_memory_service.py` (~30 тестов; полный orchestrator suite — **261 passed**, 2 skipped). Live save к MWS `qwen3-embedding-8b` может редко давать **ReadTimeout** — см. `memory_embedding_timeout_seconds`, `docs/LIVE_SMOKE.md`.</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>`classifier.py` (task type + modalities) → `router.py` (role-backed alias chain) → LiteLLM. Решение попадает в `X-GPTHub-Trace`.</t>
+          <t>`classifier.py` (task type + modalities) → `router.py` → `data/model_roles.yaml`: обычный чат → `gpt-hub-turbo` (alpha); summarization/file_analysis → **`gpt-hub-doc`** (72B) с fallback на turbo; code_help → **`gpt-hub-reasoning-or`** (coder) с fallback на turbo; vision → цепочка `gpt-hub-vision*`. Трейс: `X-GPTHub-Trace`. Канон политики: **`docs/MODEL_ROUTING_POLICY.md`**.</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>**PPTX generation**: `/pptx` или «сделай презентацию / build a deck / в формате pptx» → `task_type=PPTX_GENERATION` → `apps/orchestrator/gpthub_orchestrator/pptx_gen.py` просит `gpt-hub-strong` (glm-4.6-357b) сгенерировать JSON slide plan (с `&lt;think&gt;` CoT stripping + retry on parse failure), затем `python-pptx` собирает `.pptx` (title slide + bullet slides), файл сохраняется в `/tmp/gpthub_pptx/`, в ответ идёт markdown-ссылка на `GET /v1/files/pptx/{token}`. Один `chat.completion` на выход. 56 unit-тестов (`test_pptx_gen.py`). **Live PASS 2026-04-12**: 7-slide deck, 35 KB, download OK. Трейс: `{short_circuit:"pptx_generation", plan_model, slide_count, byte_size, plan_ms, build_ms, url}`.</t>
+          <t>**`gpthub_orchestrator/pptx/`** — intent (RU/EN + `/pptx`): `task_type=pptx`, router `pptx_slide_plan_json` (или `*_openrouter`). План слайдов: при `pptx_parallel_slide_agents_enabled` — outline LLM + параллельные per-slide агенты (семафор `pptx_slide_agents_concurrency`), иначе монолитный JSON с retry при ошибке парсинга; обрезка до `pptx_max_slides`. Сборка: `build_pptx_from_plan` (`python-pptx`, опционально шаблоны из `pptx_templates_dir` / bundled). Файл: `PptxArtifactStore` → ответ с markdown-превью + ссылка **`GET /artifacts/pptx/{id}?token=…`** (одноразовый токен, TTL `pptx_artifact_ttl_seconds`; публичный префикс `pptx_artifacts_public_base_url`). В `ingest/url_fetch.py` URL артефактов не тянутся повторно (избегаем «съедания» токена WebUI). Short-circuit в `main.py`: после memory и council, **после** image-gen. Опционально **`PPTX_PLAN_MODEL`** и алиасы `gpt-hub-pptx-*` — см. `scripts/bench_pptx_plan_models.py`. **36** тестов: `test_pptx_module.py`, `test_classifier_pptx.py`, `test_main_pptx_short_circuit.py`. В логах: `pptx_timing`, в trace — `pptx`. Живые прогоны: `docs/LIVE_SMOKE.md`.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(submission): RU headers and status hints in features xlsx
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/submission/GPTHub_features_matrix.xlsx
+++ b/docs/submission/GPTHub_features_matrix.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Features" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Матрица фич" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Справка" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,6 +28,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,9 +54,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,368 +430,612 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="88" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Row</t>
+          <t>№ ряда</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Категория</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Фича / сценарий</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>How it works in this repo</t>
+          <t>Статус (канон, EN)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Пояснение статуса (RU)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Реализация в проекте (подробно, RU)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Обязательные фичи (ряды 1–12)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Текстовый чат</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано в коде: сценарий закрыт автотестами и/или живым прогоном контракта MWS (см. docs/MWS_CATALOG.md, docs/LIVE_SMOKE.md).</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Open WebUI → orchestrator `/v1/chat/completions` → LiteLLM (по умолчанию `gpt-hub-turbo` → `mws-gpt-alpha`; другие task_type см. ряд 10). Prompt precedence + `X-GPTHub-Trace`.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Обязательные фичи (ряды 1–12)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Голосовой чат</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Implemented (UI-managed)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано через штатные настройки Open WebUI (без отдельной логики в orchestrator). Обязательны переменные окружения / тумблеры из колонки «Реализация»; без них фича не включится.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>STT/TTS Open WebUI, далее обычный orchestrator-путь. Голосовой текст проходит тот же classifier / router.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Обязательные фичи (ряды 1–12)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Генерация изображений в чате</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано в коде: сценарий закрыт автотестами и/или живым прогоном контракта MWS (см. docs/MWS_CATALOG.md, docs/LIVE_SMOKE.md).</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>`image_gen.py`: classifier ловит «нарисуй / draw / /image», orchestrator сам зовёт MWS `POST /v1/images/generations` с моделью `qwen-image`, возвращает inline markdown `![](url)` в OpenAI-совместимом ответе (json + stream). См. тесты `tests/test_image_gen.py`.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Обязательные фичи (ряды 1–12)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Аудиофайлы + автоматический ASR</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано в коде: сценарий закрыт автотестами и/или живым прогоном контракта MWS (см. docs/MWS_CATALOG.md, docs/LIVE_SMOKE.md).</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>`ingest/asr_client.py` + `Settings.resolved_asr_*()`: по умолчанию ASR идёт в MWS `whisper-medium` по тому же `MWS_GPT_API_BASE/KEY`. Можно переопределить `ORCHESTRATOR_ASR_*` для альтернативного хоста.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Обязательные фичи (ряды 1–12)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Изображения (VLM)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано в коде: сценарий закрыт автотестами и/или живым прогоном контракта MWS (см. docs/MWS_CATALOG.md, docs/LIVE_SMOKE.md).</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Ingest определяет image-part → роль `vision` → alias chain `gpt-hub-vision → vision-2 → vision-3 → vision-4 → fallback` → MWS multimodal (`qwen3-vl-30b-a3b-instruct`, `qwen2.5-vl*`, `cotype-pro-vl-32b`).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Обязательные фичи (ряды 1–12)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Файлы и ответы по содержимому</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано в коде: сценарий закрыт автотестами и/или живым прогоном контракта MWS (см. docs/MWS_CATALOG.md, docs/LIVE_SMOKE.md).</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Orchestrator `ingest/pipeline.py`: PDF через `pypdf`, DOCX/XLSX/PPTX/DOC/XLS/RTF/EPUB через `markitdown` (Microsoft), plain-text (≈30 расширений). Текст идёт как `document_text` artifact в system prompt. Тесты: `test_ingest_pdf.py`, `test_ingest_text.py`, `test_ingest_richdoc.py`.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Обязательные фичи (ряды 1–12)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Поиск в интернете</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Implemented (UI-managed)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано через штатные настройки Open WebUI (без отдельной логики в orchestrator). Обязательны переменные окружения / тумблеры из колонки «Реализация»; без них фича не включится.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Включён через Open WebUI web search (`ENABLE_WEB_SEARCH=true`, `WEB_SEARCH_ENGINE=tavily`, `TAVILY_API_KEY`). Обязательно **`BYPASS_WEB_SEARCH_EMBEDDING_AND_RETRIEVAL=true`** (или эквивалентный тумблер в Admin → Web Search): иначе WebUI пытается векторизовать сниппеты без embedding engine → ошибка и пустые источники. С bypass сниппеты **встраиваются в текст запроса** к orchestrator; **панель «источники»** может кратко показывать число находок, затем **«источники не найдены»**, потому что UI часто ждёт метаданные из пропущенного vector-пути — это **косметика**, не признак отсутствия поиска, если ответ по сути совпадает с новостями. Дальше — общий orchestrator-путь.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Обязательные фичи (ряды 1–12)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Веб-парсинг по ссылке из сообщения</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано в коде: сценарий закрыт автотестами и/или живым прогоном контракта MWS (см. docs/MWS_CATALOG.md, docs/LIVE_SMOKE.md).</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>`ingest/url_fetch.py`: детект `http(s)://` в последнем user-сообщении, fetch с таймаутом/лимитом размера, SSRF-блок приватных IP (до и после редиректов), HTML-парсер без внешних зависимостей, artifact `url_text` в system prompt. Тесты: `test_ingest_url.py` (12 тестов включая SSRF и лимиты).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Обязательные фичи (ряды 1–12)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Долгосрочная память</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>`apps/orchestrator/gpthub_orchestrator/memory/`: SQLite store (`store.py`), command parser (`commands.py`), MWS `qwen3-embedding-8b` client (`embeddings.py`), высокоуровневый сервис (`service.py`). Orchestrator ловит «запомни X / забудь X / что ты помнишь», сохраняет факты с эмбеддингом, при обычном запросе подмешивает top-K релевантных фактов как system-блок. Тесты: `test_memory_commands.py`, `test_memory_store.py`, `test_memory_service.py` (~30 тестов; полный orchestrator suite — **261 passed**, 2 skipped). Live save к MWS `qwen3-embedding-8b` может редко давать **ReadTimeout** — см. `memory_embedding_timeout_seconds`, `docs/LIVE_SMOKE.md`.</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано в коде: сценарий закрыт автотестами и/или живым прогоном контракта MWS (см. docs/MWS_CATALOG.md, docs/LIVE_SMOKE.md).</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>`apps/orchestrator/gpthub_orchestrator/memory/`: SQLite store (`store.py`), command parser (`commands.py`), MWS `qwen3-embedding-8b` client (`embeddings.py`), высокоуровневый сервис (`service.py`). Orchestrator ловит «запомни X / забудь X / что ты помнишь», сохраняет факты с эмбеддингом, при обычном запросе подмешивает top-K релевантных фактов как system-блок. Тесты: `test_memory_commands.py`, `test_memory_store.py`, `test_memory_service.py` (~30 тестов; полный набор orchestrator — **261 пройден**, 2 пропущено). Live save к MWS `qwen3-embedding-8b` может редко давать **ReadTimeout** — см. `memory_embedding_timeout_seconds`, `docs/LIVE_SMOKE.md`.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Обязательные фичи (ряды 1–12)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Автовыбор модели под задачу</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано в коде: сценарий закрыт автотестами и/или живым прогоном контракта MWS (см. docs/MWS_CATALOG.md, docs/LIVE_SMOKE.md).</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>`classifier.py` (task type + modalities) → `router.py` → `data/model_roles.yaml`: обычный чат → `gpt-hub-turbo` (alpha); summarization/file_analysis → **`gpt-hub-doc`** (72B) с fallback на turbo; code_help → **`gpt-hub-reasoning-or`** (coder) с fallback на turbo; vision → цепочка `gpt-hub-vision*`. Трейс: `X-GPTHub-Trace`. Канон политики: **`docs/MODEL_ROUTING_POLICY.md`**.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Обязательные фичи (ряды 1–12)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Ручной выбор модели</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано в коде: сценарий закрыт автотестами и/или живым прогоном контракта MWS (см. docs/MWS_CATALOG.md, docs/LIVE_SMOKE.md).</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Переключается через `ORCHESTRATOR_MODELS_CATALOG=all` + `AUTO_ROUTE_MODEL=false`. Для демо предусмотрен отдельный режим «все алиасы в dropdown WebUI».</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Обязательные фичи (ряды 1–12)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Markdown и форматированный код</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано в коде: сценарий закрыт автотестами и/или живым прогоном контракта MWS (см. docs/MWS_CATALOG.md, docs/LIVE_SMOKE.md).</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Ответ остаётся OpenAI-совместимым, Open WebUI рендерит markdown/подсветку кода штатно. `reasoning_response_filter` убирает CoT-поля, чтобы они не утекали в `content`.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Дополнительный функционал (ряды 13–15)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Deep Research / research-режим</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Implemented (WOW-1)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>**Expert Council**: `/research` или «глубокое исследование» → `task_type=DEEP_RESEARCH` → `apps/orchestrator/gpthub_orchestrator/council.py` делает параллельный fan-out в 3 MWS-модели (`gpt-hub-turbo` generalist, `gpt-hub-reasoning-or` reasoning, `gpt-hub-doc` doc-expert), каждая с собственной персоной, а затем `gpt-hub-strong` (glm-4.6-357b) синтезирует один финальный ответ в формате «суть → «что говорит совет экспертов» → практические рекомендации». CoT-очистка, partial-failure tolerant (≥2/3 веток), strong-only fallback, emergency composite если synthesis деградирует. Один `chat.completion` на выход. 29 unit-тестов (`test_council.py`) + live smoke через docker (171 s, 3/3 ветки, запись в LIVE_SMOKE.md 2026-04-11). Трейс: `{short_circuit:"expert_council", branches_ok:[...3 moderms...], synthesis_model, total_ms, fallback_used}`.</t>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано как дополнительная WOW-1 фича: не ломает единый поток чата, есть тесты и зафиксированный smoke; приоритет см. ROADMAP.md.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>**Expert Council**: `/research` или «глубокое исследование» → `task_type=DEEP_RESEARCH` → `apps/orchestrator/gpthub_orchestrator/council.py` распараллеливает запросы к **трём** MWS-моделям (`gpt-hub-turbo` generalist, `gpt-hub-reasoning-or` reasoning, `gpt-hub-doc` doc-expert), у каждой своя персона, затем `gpt-hub-strong` (glm-4.6-357b) **синтезирует один** финальный ответ: «суть → что говорит совет экспертов → практические рекомендации». Очистка цепочки рассуждений (CoT), устойчивость к частичным сбоям (нужно ≥2 из 3 веток), запасной путь только на strong-модель, аварийный составной ответ при деградации синтеза. Снаружи — один ответ `chat.completion`. **29** unit-тестов (`test_council.py`) + live smoke в docker (~171 с, 3/3 ветки, запись в `LIVE_SMOKE.md` 2026-04-11). В трейсе: `short_circuit: expert_council`, ветки, модель синтеза, время, использован ли fallback.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Дополнительный функционал (ряды 13–15)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Генерация презентаций</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Implemented (WOW-3)</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано как дополнительная WOW-3 фича: не ломает единый поток чата, есть тесты и записи в LIVE_SMOKE.md; приоритет см. ROADMAP.md.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>**`gpthub_orchestrator/pptx/`** — intent (RU/EN + `/pptx`): `task_type=pptx`, router `pptx_slide_plan_json` (или `*_openrouter`). План слайдов: при `pptx_parallel_slide_agents_enabled` — outline LLM + параллельные per-slide агенты (семафор `pptx_slide_agents_concurrency`), иначе монолитный JSON с retry при ошибке парсинга; обрезка до `pptx_max_slides`. Сборка: `build_pptx_from_plan` (`python-pptx`, опционально шаблоны из `pptx_templates_dir` / bundled). Файл: `PptxArtifactStore` → ответ с markdown-превью + ссылка **`GET /artifacts/pptx/{id}?token=…`** (одноразовый токен, TTL `pptx_artifact_ttl_seconds`; публичный префикс `pptx_artifacts_public_base_url`). В `ingest/url_fetch.py` URL артефактов не тянутся повторно (избегаем «съедания» токена WebUI). Short-circuit в `main.py`: после memory и council, **после** image-gen. Опционально **`PPTX_PLAN_MODEL`** и алиасы `gpt-hub-pptx-*` — см. `scripts/bench_pptx_plan_models.py`. **36** тестов: `test_pptx_module.py`, `test_classifier_pptx.py`, `test_main_pptx_short_circuit.py`. В логах: `pptx_timing`, в trace — `pptx`. Живые прогоны: `docs/LIVE_SMOKE.md`.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Дополнительный функционал (ряды 13–15)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Другой доп. функционал</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>**`X-GPTHub-Trace`** — production-grade наблюдаемость: routing decision, model chain, fallback attempts, ingest artifacts, classifier source, prompt version, server clock, ingest latency. Header не утекает в `content`. На защите показывается в DevTools.</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано в коде: сценарий закрыт автотестами и/или живым прогоном контракта MWS (см. docs/MWS_CATALOG.md, docs/LIVE_SMOKE.md).</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>**`X-GPTHub-Trace`** — наблюдаемость уровня продакшена: решение маршрутизатора, цепочка моделей, попытки fallback, артефакты ingest, источник решения классификатора, версия промпта, время сервера, задержки ingest. Заголовок ответа **не** попадает в текст `content` для пользователя; на защите удобно смотреть в DevTools → Network.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Этот файл собран из FEATURE_MATRIX.md (корень репозитория). Пересборка: uv run --with openpyxl python scripts/build_features_xlsx.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Код статуса (канон)</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Расшифровка по-русски</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Код в репозитории, тесты проходят, путь подтверждён контрактом MWS или unit/integration тестом.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Implemented (UI-managed)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Работает через встроенные возможности Open WebUI; в orchestrator отдельной реализации нет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Implemented (WOW-1) / (WOW-3)</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Реализовано как дополнительный WOW-сценарий; требования к доказательствам те же, что у Implemented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Wired, pending live smoke</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Код есть, нужен сквозной прогон через docker-stack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Сценарий закрыт не полностью.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Не реализовано; отложено.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>